<commit_message>
chore: update Fanqie male rankings
</commit_message>
<xml_diff>
--- a/data/持续收益潜力作品.xlsx
+++ b/data/持续收益潜力作品.xlsx
@@ -10,19 +10,19 @@
     <sheet name="作品数据" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">作品数据!$A$4:$O$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">作品数据!$A$4:$O$54</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="68">
   <si>
     <t>持续收益潜力作品</t>
   </si>
   <si>
-    <t>生成时间：2026-09-15T04:35:52+00:00。候选名单仅依据公开榜单的连续出现、在读规模和在读变化筛选，不代表真实稿费、订阅收入或平台结算。</t>
+    <t>生成时间：2026-09-16T04:31:27+00:00。候选名单仅依据公开榜单的连续出现、在读规模和在读变化筛选，不代表真实稿费、订阅收入或平台结算。</t>
   </si>
   <si>
     <t>作品名</t>
@@ -68,13 +68,170 @@
   </si>
   <si>
     <t>达标日期列表</t>
+  </si>
+  <si>
+    <t>点子王行动哥随便弟，三人行很刑</t>
+  </si>
+  <si>
+    <t>打开作品</t>
+  </si>
+  <si>
+    <t>规则怪谈：无所谓，系统会出手</t>
+  </si>
+  <si>
+    <t>游走神话时代，开局拜师道门天师</t>
+  </si>
+  <si>
+    <t>武侠网游，开局三个神级词条</t>
+  </si>
+  <si>
+    <t>无声1937</t>
+  </si>
+  <si>
+    <t>火影：扉间问谁断后，我当三代！</t>
+  </si>
+  <si>
+    <t>刚穿越洪荒，就要被弑神枪钉死了</t>
+  </si>
+  <si>
+    <t>魏家孽种成首辅，全族跪求我认祖</t>
+  </si>
+  <si>
+    <t>系统想害我，我选择上交国家</t>
+  </si>
+  <si>
+    <t>穿越成国公，咋就是封建余孽了？</t>
+  </si>
+  <si>
+    <t>我一写网文的，你让我混娱乐圈？</t>
+  </si>
+  <si>
+    <t>西游：大圣闹地府！始皇长生啦</t>
+  </si>
+  <si>
+    <t>死刑当天，修仙者夺舍了我</t>
+  </si>
+  <si>
+    <t>我都永生了，会亿点技能很合理吧</t>
+  </si>
+  <si>
+    <t>人在高中，香火证道什么鬼？</t>
+  </si>
+  <si>
+    <t>综漫：表白被拒就变强？</t>
+  </si>
+  <si>
+    <t>无敌江湖后，我隐退于世</t>
+  </si>
+  <si>
+    <t>奥特：天蝎座第一道光</t>
+  </si>
+  <si>
+    <t>重生八零渔村，带仨前妻赶海暴富</t>
+  </si>
+  <si>
+    <t>无职：验牌洛琪希，牌没有问题？</t>
+  </si>
+  <si>
+    <t>末世选择：开局一亿只美洲大蠊</t>
+  </si>
+  <si>
+    <t>末世：我开局拥有一艘驱逐舰</t>
+  </si>
+  <si>
+    <t>从金丹仙族开始的老祖之路！</t>
+  </si>
+  <si>
+    <t>一心求死，反倒成为千古一帝？</t>
+  </si>
+  <si>
+    <t>娱乐圈在线吃瓜，嘎嘎吃瓜嘎嘎香</t>
+  </si>
+  <si>
+    <t>洪荒：我十凶天角蚁，躺平就变强</t>
+  </si>
+  <si>
+    <t>斩神师兄太我清道德天尊社恐反差</t>
+  </si>
+  <si>
+    <t>从零开始，打造华夏首支特种部队</t>
+  </si>
+  <si>
+    <t>要当总统了，你跟我说系统来了？</t>
+  </si>
+  <si>
+    <t>模拟未来：我是叛徒？请世家赴死</t>
+  </si>
+  <si>
+    <t>西游降临：开局拜师通天教主！</t>
+  </si>
+  <si>
+    <t>打卡双人骑行圈，开局拿捏假名媛</t>
+  </si>
+  <si>
+    <t>一毛一天修为，我靠直播氪穿宇宙</t>
+  </si>
+  <si>
+    <t>诡异世界，我的神通无限升级！</t>
+  </si>
+  <si>
+    <t>穿越黄毛，女主们把我当白月光了</t>
+  </si>
+  <si>
+    <t>灵气复苏？前世女帝老婆也复苏了</t>
+  </si>
+  <si>
+    <t>我有一个女鬼催眠APP</t>
+  </si>
+  <si>
+    <t>别人穿四合院，我为啥上战场</t>
+  </si>
+  <si>
+    <t>秦始皇：朕有华夏全明星阵容</t>
+  </si>
+  <si>
+    <t>天渊</t>
+  </si>
+  <si>
+    <t>玄幻：多管闲事，成人间武圣</t>
+  </si>
+  <si>
+    <t>不是，啥叫世界会自主更新版本？</t>
+  </si>
+  <si>
+    <t>分手后，她们变得不对劲了！</t>
+  </si>
+  <si>
+    <t>刚上大一，哪来五个病娇未婚妻？</t>
+  </si>
+  <si>
+    <t>老师，男生也能报考魔女学院吗？</t>
+  </si>
+  <si>
+    <t>青梅是天命之女？可我既是天命！</t>
+  </si>
+  <si>
+    <t>名义，汉东刘长生，谁与争锋！</t>
+  </si>
+  <si>
+    <t>爱情公寓：开局拿下林妙妙</t>
+  </si>
+  <si>
+    <t>楼层求生：从垃圾场开始变废为宝</t>
+  </si>
+  <si>
+    <t>列车求生：我的乘员提供暴击结算</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="4">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="#,##0.0"/>
+    <numFmt numFmtId="165" formatCode="#,##0"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -105,6 +262,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0563C1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -126,7 +291,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -149,11 +314,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE6E6E6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE6E6E6"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE6E6E6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE6E6E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -163,6 +343,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -458,7 +650,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -561,12 +753,1716 @@
         <v>16</v>
       </c>
     </row>
+    <row r="5" spans="1:15">
+      <c r="A5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5">
+        <v>100</v>
+      </c>
+      <c r="D5" s="4"/>
+      <c r="E5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="7">
+        <v>848000</v>
+      </c>
+      <c r="G5" s="7">
+        <v>81000</v>
+      </c>
+      <c r="H5" s="7">
+        <v>3</v>
+      </c>
+      <c r="I5" s="7">
+        <v>86000</v>
+      </c>
+      <c r="J5" s="5">
+        <v>85.5</v>
+      </c>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="5"/>
+      <c r="O5" s="4"/>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="A6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5">
+        <v>84.59999999999999</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="7">
+        <v>1549000</v>
+      </c>
+      <c r="G6" s="7">
+        <v>67000</v>
+      </c>
+      <c r="H6" s="7">
+        <v>3</v>
+      </c>
+      <c r="I6" s="7">
+        <v>74000</v>
+      </c>
+      <c r="J6" s="5">
+        <v>74</v>
+      </c>
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="5"/>
+      <c r="O6" s="4"/>
+    </row>
+    <row r="7" spans="1:15">
+      <c r="A7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5">
+        <v>100</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="7">
+        <v>246000</v>
+      </c>
+      <c r="G7" s="7">
+        <v>41000</v>
+      </c>
+      <c r="H7" s="7">
+        <v>3</v>
+      </c>
+      <c r="I7" s="7">
+        <v>39500</v>
+      </c>
+      <c r="J7" s="5">
+        <v>73.90000000000001</v>
+      </c>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="5"/>
+      <c r="O7" s="4"/>
+    </row>
+    <row r="8" spans="1:15">
+      <c r="A8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5">
+        <v>100</v>
+      </c>
+      <c r="D8" s="4"/>
+      <c r="E8" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="7">
+        <v>155000</v>
+      </c>
+      <c r="G8" s="7">
+        <v>32000</v>
+      </c>
+      <c r="H8" s="7">
+        <v>3</v>
+      </c>
+      <c r="I8" s="7">
+        <v>29000</v>
+      </c>
+      <c r="J8" s="5">
+        <v>71.2</v>
+      </c>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="5"/>
+      <c r="O8" s="4"/>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5">
+        <v>89.5</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="7">
+        <v>384000</v>
+      </c>
+      <c r="G9" s="7">
+        <v>40000</v>
+      </c>
+      <c r="H9" s="7">
+        <v>3</v>
+      </c>
+      <c r="I9" s="7">
+        <v>43500</v>
+      </c>
+      <c r="J9" s="5">
+        <v>69.09999999999999</v>
+      </c>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="4"/>
+    </row>
+    <row r="10" spans="1:15">
+      <c r="A10" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5">
+        <v>95.90000000000001</v>
+      </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="7">
+        <v>344000</v>
+      </c>
+      <c r="G10" s="7">
+        <v>26000</v>
+      </c>
+      <c r="H10" s="7">
+        <v>3</v>
+      </c>
+      <c r="I10" s="7">
+        <v>26000</v>
+      </c>
+      <c r="J10" s="5">
+        <v>68.2</v>
+      </c>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="4"/>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="A11" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5">
+        <v>100</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11" s="7">
+        <v>131000</v>
+      </c>
+      <c r="G11" s="7">
+        <v>18000</v>
+      </c>
+      <c r="H11" s="7">
+        <v>3</v>
+      </c>
+      <c r="I11" s="7">
+        <v>13000</v>
+      </c>
+      <c r="J11" s="5">
+        <v>67.2</v>
+      </c>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="5"/>
+      <c r="O11" s="4"/>
+    </row>
+    <row r="12" spans="1:15">
+      <c r="A12" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5">
+        <v>88.09999999999999</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" s="7">
+        <v>421000</v>
+      </c>
+      <c r="G12" s="7">
+        <v>68000</v>
+      </c>
+      <c r="H12" s="7">
+        <v>3</v>
+      </c>
+      <c r="I12" s="7">
+        <v>37500</v>
+      </c>
+      <c r="J12" s="5">
+        <v>66.8</v>
+      </c>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="5"/>
+      <c r="O12" s="4"/>
+    </row>
+    <row r="13" spans="1:15">
+      <c r="A13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5">
+        <v>83</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" s="7">
+        <v>1517000</v>
+      </c>
+      <c r="G13" s="7">
+        <v>31000</v>
+      </c>
+      <c r="H13" s="7">
+        <v>3</v>
+      </c>
+      <c r="I13" s="7">
+        <v>45500</v>
+      </c>
+      <c r="J13" s="5">
+        <v>66</v>
+      </c>
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="4"/>
+    </row>
+    <row r="14" spans="1:15">
+      <c r="A14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5">
+        <v>99</v>
+      </c>
+      <c r="D14" s="4"/>
+      <c r="E14" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" s="7">
+        <v>220000</v>
+      </c>
+      <c r="G14" s="7">
+        <v>24000</v>
+      </c>
+      <c r="H14" s="7">
+        <v>3</v>
+      </c>
+      <c r="I14" s="7">
+        <v>6000</v>
+      </c>
+      <c r="J14" s="5">
+        <v>65</v>
+      </c>
+      <c r="K14" s="4"/>
+      <c r="L14" s="4"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="4"/>
+    </row>
+    <row r="15" spans="1:15">
+      <c r="A15" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5">
+        <v>83</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" s="7">
+        <v>894000</v>
+      </c>
+      <c r="G15" s="7">
+        <v>35000</v>
+      </c>
+      <c r="H15" s="7">
+        <v>3</v>
+      </c>
+      <c r="I15" s="7">
+        <v>40500</v>
+      </c>
+      <c r="J15" s="5">
+        <v>64.8</v>
+      </c>
+      <c r="K15" s="4"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="7"/>
+      <c r="N15" s="5"/>
+      <c r="O15" s="4"/>
+    </row>
+    <row r="16" spans="1:15">
+      <c r="A16" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5">
+        <v>91.40000000000001</v>
+      </c>
+      <c r="D16" s="4"/>
+      <c r="E16" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F16" s="7">
+        <v>129000</v>
+      </c>
+      <c r="G16" s="7">
+        <v>22000</v>
+      </c>
+      <c r="H16" s="7">
+        <v>3</v>
+      </c>
+      <c r="I16" s="7">
+        <v>20500</v>
+      </c>
+      <c r="J16" s="5">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="5"/>
+      <c r="O16" s="4"/>
+    </row>
+    <row r="17" spans="1:15">
+      <c r="A17" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5">
+        <v>86.8</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" s="7">
+        <v>275000</v>
+      </c>
+      <c r="G17" s="7">
+        <v>35000</v>
+      </c>
+      <c r="H17" s="7">
+        <v>3</v>
+      </c>
+      <c r="I17" s="7">
+        <v>29000</v>
+      </c>
+      <c r="J17" s="5">
+        <v>64</v>
+      </c>
+      <c r="K17" s="4"/>
+      <c r="L17" s="4"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="5"/>
+      <c r="O17" s="4"/>
+    </row>
+    <row r="18" spans="1:15">
+      <c r="A18" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5">
+        <v>82.8</v>
+      </c>
+      <c r="D18" s="4"/>
+      <c r="E18" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" s="7">
+        <v>403000</v>
+      </c>
+      <c r="G18" s="7">
+        <v>44000</v>
+      </c>
+      <c r="H18" s="7">
+        <v>3</v>
+      </c>
+      <c r="I18" s="7">
+        <v>35500</v>
+      </c>
+      <c r="J18" s="5">
+        <v>63.4</v>
+      </c>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="5"/>
+      <c r="O18" s="4"/>
+    </row>
+    <row r="19" spans="1:15">
+      <c r="A19" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5">
+        <v>89.59999999999999</v>
+      </c>
+      <c r="D19" s="4"/>
+      <c r="E19" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F19" s="7">
+        <v>199000</v>
+      </c>
+      <c r="G19" s="7">
+        <v>15000</v>
+      </c>
+      <c r="H19" s="7">
+        <v>3</v>
+      </c>
+      <c r="I19" s="7">
+        <v>19500</v>
+      </c>
+      <c r="J19" s="5">
+        <v>63.2</v>
+      </c>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="7"/>
+      <c r="N19" s="5"/>
+      <c r="O19" s="4"/>
+    </row>
+    <row r="20" spans="1:15">
+      <c r="A20" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5">
+        <v>92.8</v>
+      </c>
+      <c r="D20" s="4"/>
+      <c r="E20" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" s="7">
+        <v>181000</v>
+      </c>
+      <c r="G20" s="7">
+        <v>15000</v>
+      </c>
+      <c r="H20" s="7">
+        <v>3</v>
+      </c>
+      <c r="I20" s="7">
+        <v>12500</v>
+      </c>
+      <c r="J20" s="5">
+        <v>63.2</v>
+      </c>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="7"/>
+      <c r="N20" s="5"/>
+      <c r="O20" s="4"/>
+    </row>
+    <row r="21" spans="1:15">
+      <c r="A21" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5">
+        <v>93.59999999999999</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F21" s="7">
+        <v>105000</v>
+      </c>
+      <c r="G21" s="7">
+        <v>9000</v>
+      </c>
+      <c r="H21" s="7">
+        <v>3</v>
+      </c>
+      <c r="I21" s="7">
+        <v>10000</v>
+      </c>
+      <c r="J21" s="5">
+        <v>63</v>
+      </c>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="7"/>
+      <c r="N21" s="5"/>
+      <c r="O21" s="4"/>
+    </row>
+    <row r="22" spans="1:15">
+      <c r="A22" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5">
+        <v>83.2</v>
+      </c>
+      <c r="D22" s="4"/>
+      <c r="E22" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F22" s="7">
+        <v>282000</v>
+      </c>
+      <c r="G22" s="7">
+        <v>20000</v>
+      </c>
+      <c r="H22" s="7">
+        <v>3</v>
+      </c>
+      <c r="I22" s="7">
+        <v>32000</v>
+      </c>
+      <c r="J22" s="5">
+        <v>62.8</v>
+      </c>
+      <c r="K22" s="4"/>
+      <c r="L22" s="4"/>
+      <c r="M22" s="7"/>
+      <c r="N22" s="5"/>
+      <c r="O22" s="4"/>
+    </row>
+    <row r="23" spans="1:15">
+      <c r="A23" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5">
+        <v>91.8</v>
+      </c>
+      <c r="D23" s="4"/>
+      <c r="E23" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" s="7">
+        <v>162000</v>
+      </c>
+      <c r="G23" s="7">
+        <v>10000</v>
+      </c>
+      <c r="H23" s="7">
+        <v>3</v>
+      </c>
+      <c r="I23" s="7">
+        <v>12000</v>
+      </c>
+      <c r="J23" s="5">
+        <v>62.5</v>
+      </c>
+      <c r="K23" s="4"/>
+      <c r="L23" s="4"/>
+      <c r="M23" s="7"/>
+      <c r="N23" s="5"/>
+      <c r="O23" s="4"/>
+    </row>
+    <row r="24" spans="1:15">
+      <c r="A24" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5">
+        <v>85.7</v>
+      </c>
+      <c r="D24" s="4"/>
+      <c r="E24" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F24" s="7">
+        <v>213000</v>
+      </c>
+      <c r="G24" s="7">
+        <v>22000</v>
+      </c>
+      <c r="H24" s="7">
+        <v>3</v>
+      </c>
+      <c r="I24" s="7">
+        <v>23500</v>
+      </c>
+      <c r="J24" s="5">
+        <v>62</v>
+      </c>
+      <c r="K24" s="4"/>
+      <c r="L24" s="4"/>
+      <c r="M24" s="7"/>
+      <c r="N24" s="5"/>
+      <c r="O24" s="4"/>
+    </row>
+    <row r="25" spans="1:15">
+      <c r="A25" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25" s="5"/>
+      <c r="C25" s="5">
+        <v>88.8</v>
+      </c>
+      <c r="D25" s="4"/>
+      <c r="E25" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F25" s="7">
+        <v>423000</v>
+      </c>
+      <c r="G25" s="7">
+        <v>3000</v>
+      </c>
+      <c r="H25" s="7">
+        <v>3</v>
+      </c>
+      <c r="I25" s="7">
+        <v>16000</v>
+      </c>
+      <c r="J25" s="5">
+        <v>61.8</v>
+      </c>
+      <c r="K25" s="4"/>
+      <c r="L25" s="4"/>
+      <c r="M25" s="7"/>
+      <c r="N25" s="5"/>
+      <c r="O25" s="4"/>
+    </row>
+    <row r="26" spans="1:15">
+      <c r="A26" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" s="5"/>
+      <c r="C26" s="5">
+        <v>90.8</v>
+      </c>
+      <c r="D26" s="4"/>
+      <c r="E26" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" s="7">
+        <v>173000</v>
+      </c>
+      <c r="G26" s="7">
+        <v>9000</v>
+      </c>
+      <c r="H26" s="7">
+        <v>3</v>
+      </c>
+      <c r="I26" s="7">
+        <v>10500</v>
+      </c>
+      <c r="J26" s="5">
+        <v>61.6</v>
+      </c>
+      <c r="K26" s="4"/>
+      <c r="L26" s="4"/>
+      <c r="M26" s="7"/>
+      <c r="N26" s="5"/>
+      <c r="O26" s="4"/>
+    </row>
+    <row r="27" spans="1:15">
+      <c r="A27" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F27" s="7">
+        <v>631000</v>
+      </c>
+      <c r="G27" s="7">
+        <v>21000</v>
+      </c>
+      <c r="H27" s="7">
+        <v>3</v>
+      </c>
+      <c r="I27" s="7">
+        <v>29500</v>
+      </c>
+      <c r="J27" s="5">
+        <v>61.3</v>
+      </c>
+      <c r="K27" s="4"/>
+      <c r="L27" s="4"/>
+      <c r="M27" s="7"/>
+      <c r="N27" s="5"/>
+      <c r="O27" s="4"/>
+    </row>
+    <row r="28" spans="1:15">
+      <c r="A28" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" s="5"/>
+      <c r="C28" s="5">
+        <v>83.3</v>
+      </c>
+      <c r="D28" s="4"/>
+      <c r="E28" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F28" s="7">
+        <v>448000</v>
+      </c>
+      <c r="G28" s="7">
+        <v>25000</v>
+      </c>
+      <c r="H28" s="7">
+        <v>3</v>
+      </c>
+      <c r="I28" s="7">
+        <v>26000</v>
+      </c>
+      <c r="J28" s="5">
+        <v>61.3</v>
+      </c>
+      <c r="K28" s="4"/>
+      <c r="L28" s="4"/>
+      <c r="M28" s="7"/>
+      <c r="N28" s="5"/>
+      <c r="O28" s="4"/>
+    </row>
+    <row r="29" spans="1:15">
+      <c r="A29" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5">
+        <v>77.7</v>
+      </c>
+      <c r="D29" s="4"/>
+      <c r="E29" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F29" s="7">
+        <v>430000</v>
+      </c>
+      <c r="G29" s="7">
+        <v>25000</v>
+      </c>
+      <c r="H29" s="7">
+        <v>3</v>
+      </c>
+      <c r="I29" s="7">
+        <v>37500</v>
+      </c>
+      <c r="J29" s="5">
+        <v>61.1</v>
+      </c>
+      <c r="K29" s="4"/>
+      <c r="L29" s="4"/>
+      <c r="M29" s="7"/>
+      <c r="N29" s="5"/>
+      <c r="O29" s="4"/>
+    </row>
+    <row r="30" spans="1:15">
+      <c r="A30" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="5"/>
+      <c r="C30" s="5">
+        <v>90</v>
+      </c>
+      <c r="D30" s="4"/>
+      <c r="E30" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F30" s="7">
+        <v>166000</v>
+      </c>
+      <c r="G30" s="7">
+        <v>10000</v>
+      </c>
+      <c r="H30" s="7">
+        <v>3</v>
+      </c>
+      <c r="I30" s="7">
+        <v>10500</v>
+      </c>
+      <c r="J30" s="5">
+        <v>61.1</v>
+      </c>
+      <c r="K30" s="4"/>
+      <c r="L30" s="4"/>
+      <c r="M30" s="7"/>
+      <c r="N30" s="5"/>
+      <c r="O30" s="4"/>
+    </row>
+    <row r="31" spans="1:15">
+      <c r="A31" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5">
+        <v>88.5</v>
+      </c>
+      <c r="D31" s="4"/>
+      <c r="E31" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F31" s="7">
+        <v>184000</v>
+      </c>
+      <c r="G31" s="7">
+        <v>11000</v>
+      </c>
+      <c r="H31" s="7">
+        <v>3</v>
+      </c>
+      <c r="I31" s="7">
+        <v>11500</v>
+      </c>
+      <c r="J31" s="5">
+        <v>60.6</v>
+      </c>
+      <c r="K31" s="4"/>
+      <c r="L31" s="4"/>
+      <c r="M31" s="7"/>
+      <c r="N31" s="5"/>
+      <c r="O31" s="4"/>
+    </row>
+    <row r="32" spans="1:15">
+      <c r="A32" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B32" s="5"/>
+      <c r="C32" s="5">
+        <v>86.3</v>
+      </c>
+      <c r="D32" s="4"/>
+      <c r="E32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F32" s="7">
+        <v>189000</v>
+      </c>
+      <c r="G32" s="7">
+        <v>17000</v>
+      </c>
+      <c r="H32" s="7">
+        <v>3</v>
+      </c>
+      <c r="I32" s="7">
+        <v>16000</v>
+      </c>
+      <c r="J32" s="5">
+        <v>60.5</v>
+      </c>
+      <c r="K32" s="4"/>
+      <c r="L32" s="4"/>
+      <c r="M32" s="7"/>
+      <c r="N32" s="5"/>
+      <c r="O32" s="4"/>
+    </row>
+    <row r="33" spans="1:15">
+      <c r="A33" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B33" s="5"/>
+      <c r="C33" s="5">
+        <v>90</v>
+      </c>
+      <c r="D33" s="4"/>
+      <c r="E33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F33" s="7">
+        <v>147000</v>
+      </c>
+      <c r="G33" s="7">
+        <v>7000</v>
+      </c>
+      <c r="H33" s="7">
+        <v>3</v>
+      </c>
+      <c r="I33" s="7">
+        <v>7000</v>
+      </c>
+      <c r="J33" s="5">
+        <v>60.3</v>
+      </c>
+      <c r="K33" s="4"/>
+      <c r="L33" s="4"/>
+      <c r="M33" s="7"/>
+      <c r="N33" s="5"/>
+      <c r="O33" s="4"/>
+    </row>
+    <row r="34" spans="1:15">
+      <c r="A34" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B34" s="5"/>
+      <c r="C34" s="5">
+        <v>89.59999999999999</v>
+      </c>
+      <c r="D34" s="4"/>
+      <c r="E34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F34" s="7">
+        <v>103000</v>
+      </c>
+      <c r="G34" s="7">
+        <v>9000</v>
+      </c>
+      <c r="H34" s="7">
+        <v>3</v>
+      </c>
+      <c r="I34" s="7">
+        <v>8000</v>
+      </c>
+      <c r="J34" s="5">
+        <v>60.3</v>
+      </c>
+      <c r="K34" s="4"/>
+      <c r="L34" s="4"/>
+      <c r="M34" s="7"/>
+      <c r="N34" s="5"/>
+      <c r="O34" s="4"/>
+    </row>
+    <row r="35" spans="1:15">
+      <c r="A35" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B35" s="5"/>
+      <c r="C35" s="5">
+        <v>80.2</v>
+      </c>
+      <c r="D35" s="4"/>
+      <c r="E35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F35" s="7">
+        <v>903000</v>
+      </c>
+      <c r="G35" s="7">
+        <v>26000</v>
+      </c>
+      <c r="H35" s="7">
+        <v>3</v>
+      </c>
+      <c r="I35" s="7">
+        <v>28500</v>
+      </c>
+      <c r="J35" s="5">
+        <v>60.2</v>
+      </c>
+      <c r="K35" s="4"/>
+      <c r="L35" s="4"/>
+      <c r="M35" s="7"/>
+      <c r="N35" s="5"/>
+      <c r="O35" s="4"/>
+    </row>
+    <row r="36" spans="1:15">
+      <c r="A36" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B36" s="5"/>
+      <c r="C36" s="5">
+        <v>87.5</v>
+      </c>
+      <c r="D36" s="4"/>
+      <c r="E36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F36" s="7">
+        <v>454000</v>
+      </c>
+      <c r="G36" s="7">
+        <v>0</v>
+      </c>
+      <c r="H36" s="7">
+        <v>3</v>
+      </c>
+      <c r="I36" s="7">
+        <v>11500</v>
+      </c>
+      <c r="J36" s="5">
+        <v>60</v>
+      </c>
+      <c r="K36" s="4"/>
+      <c r="L36" s="4"/>
+      <c r="M36" s="7"/>
+      <c r="N36" s="5"/>
+      <c r="O36" s="4"/>
+    </row>
+    <row r="37" spans="1:15">
+      <c r="A37" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B37" s="5"/>
+      <c r="C37" s="5">
+        <v>88.5</v>
+      </c>
+      <c r="D37" s="4"/>
+      <c r="E37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F37" s="7">
+        <v>118000</v>
+      </c>
+      <c r="G37" s="7">
+        <v>8000</v>
+      </c>
+      <c r="H37" s="7">
+        <v>3</v>
+      </c>
+      <c r="I37" s="7">
+        <v>7500</v>
+      </c>
+      <c r="J37" s="5">
+        <v>59.6</v>
+      </c>
+      <c r="K37" s="4"/>
+      <c r="L37" s="4"/>
+      <c r="M37" s="7"/>
+      <c r="N37" s="5"/>
+      <c r="O37" s="4"/>
+    </row>
+    <row r="38" spans="1:15">
+      <c r="A38" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" s="5"/>
+      <c r="C38" s="5">
+        <v>86.7</v>
+      </c>
+      <c r="D38" s="4"/>
+      <c r="E38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F38" s="7">
+        <v>122000</v>
+      </c>
+      <c r="G38" s="7">
+        <v>9000</v>
+      </c>
+      <c r="H38" s="7">
+        <v>3</v>
+      </c>
+      <c r="I38" s="7">
+        <v>11000</v>
+      </c>
+      <c r="J38" s="5">
+        <v>59.4</v>
+      </c>
+      <c r="K38" s="4"/>
+      <c r="L38" s="4"/>
+      <c r="M38" s="7"/>
+      <c r="N38" s="5"/>
+      <c r="O38" s="4"/>
+    </row>
+    <row r="39" spans="1:15">
+      <c r="A39" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B39" s="5"/>
+      <c r="C39" s="5">
+        <v>87.2</v>
+      </c>
+      <c r="D39" s="4"/>
+      <c r="E39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F39" s="7">
+        <v>130000</v>
+      </c>
+      <c r="G39" s="7">
+        <v>10000</v>
+      </c>
+      <c r="H39" s="7">
+        <v>3</v>
+      </c>
+      <c r="I39" s="7">
+        <v>9500</v>
+      </c>
+      <c r="J39" s="5">
+        <v>59.3</v>
+      </c>
+      <c r="K39" s="4"/>
+      <c r="L39" s="4"/>
+      <c r="M39" s="7"/>
+      <c r="N39" s="5"/>
+      <c r="O39" s="4"/>
+    </row>
+    <row r="40" spans="1:15">
+      <c r="A40" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5">
+        <v>81.2</v>
+      </c>
+      <c r="D40" s="4"/>
+      <c r="E40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F40" s="7">
+        <v>244000</v>
+      </c>
+      <c r="G40" s="7">
+        <v>19000</v>
+      </c>
+      <c r="H40" s="7">
+        <v>3</v>
+      </c>
+      <c r="I40" s="7">
+        <v>22000</v>
+      </c>
+      <c r="J40" s="5">
+        <v>59.2</v>
+      </c>
+      <c r="K40" s="4"/>
+      <c r="L40" s="4"/>
+      <c r="M40" s="7"/>
+      <c r="N40" s="5"/>
+      <c r="O40" s="4"/>
+    </row>
+    <row r="41" spans="1:15">
+      <c r="A41" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41" s="5"/>
+      <c r="C41" s="5">
+        <v>87.90000000000001</v>
+      </c>
+      <c r="D41" s="4"/>
+      <c r="E41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F41" s="7">
+        <v>314000</v>
+      </c>
+      <c r="G41" s="7">
+        <v>4000</v>
+      </c>
+      <c r="H41" s="7">
+        <v>3</v>
+      </c>
+      <c r="I41" s="7">
+        <v>7000</v>
+      </c>
+      <c r="J41" s="5">
+        <v>59.1</v>
+      </c>
+      <c r="K41" s="4"/>
+      <c r="L41" s="4"/>
+      <c r="M41" s="7"/>
+      <c r="N41" s="5"/>
+      <c r="O41" s="4"/>
+    </row>
+    <row r="42" spans="1:15">
+      <c r="A42" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B42" s="5"/>
+      <c r="C42" s="5">
+        <v>81.5</v>
+      </c>
+      <c r="D42" s="4"/>
+      <c r="E42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F42" s="7">
+        <v>375000</v>
+      </c>
+      <c r="G42" s="7">
+        <v>16000</v>
+      </c>
+      <c r="H42" s="7">
+        <v>3</v>
+      </c>
+      <c r="I42" s="7">
+        <v>20500</v>
+      </c>
+      <c r="J42" s="5">
+        <v>59</v>
+      </c>
+      <c r="K42" s="4"/>
+      <c r="L42" s="4"/>
+      <c r="M42" s="7"/>
+      <c r="N42" s="5"/>
+      <c r="O42" s="4"/>
+    </row>
+    <row r="43" spans="1:15">
+      <c r="A43" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B43" s="5"/>
+      <c r="C43" s="5">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="D43" s="4"/>
+      <c r="E43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F43" s="7">
+        <v>280000</v>
+      </c>
+      <c r="G43" s="7">
+        <v>20000</v>
+      </c>
+      <c r="H43" s="7">
+        <v>3</v>
+      </c>
+      <c r="I43" s="7">
+        <v>20500</v>
+      </c>
+      <c r="J43" s="5">
+        <v>59</v>
+      </c>
+      <c r="K43" s="4"/>
+      <c r="L43" s="4"/>
+      <c r="M43" s="7"/>
+      <c r="N43" s="5"/>
+      <c r="O43" s="4"/>
+    </row>
+    <row r="44" spans="1:15">
+      <c r="A44" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B44" s="5"/>
+      <c r="C44" s="5">
+        <v>82</v>
+      </c>
+      <c r="D44" s="4"/>
+      <c r="E44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F44" s="7">
+        <v>1232000</v>
+      </c>
+      <c r="G44" s="7">
+        <v>19000</v>
+      </c>
+      <c r="H44" s="7">
+        <v>3</v>
+      </c>
+      <c r="I44" s="7">
+        <v>19000</v>
+      </c>
+      <c r="J44" s="5">
+        <v>58.9</v>
+      </c>
+      <c r="K44" s="4"/>
+      <c r="L44" s="4"/>
+      <c r="M44" s="7"/>
+      <c r="N44" s="5"/>
+      <c r="O44" s="4"/>
+    </row>
+    <row r="45" spans="1:15">
+      <c r="A45" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B45" s="5"/>
+      <c r="C45" s="5">
+        <v>75.2</v>
+      </c>
+      <c r="D45" s="4"/>
+      <c r="E45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F45" s="7">
+        <v>336000</v>
+      </c>
+      <c r="G45" s="7">
+        <v>33000</v>
+      </c>
+      <c r="H45" s="7">
+        <v>3</v>
+      </c>
+      <c r="I45" s="7">
+        <v>34000</v>
+      </c>
+      <c r="J45" s="5">
+        <v>58.9</v>
+      </c>
+      <c r="K45" s="4"/>
+      <c r="L45" s="4"/>
+      <c r="M45" s="7"/>
+      <c r="N45" s="5"/>
+      <c r="O45" s="4"/>
+    </row>
+    <row r="46" spans="1:15">
+      <c r="A46" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B46" s="5"/>
+      <c r="C46" s="5">
+        <v>86.09999999999999</v>
+      </c>
+      <c r="D46" s="4"/>
+      <c r="E46" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F46" s="7">
+        <v>135000</v>
+      </c>
+      <c r="G46" s="7">
+        <v>7000</v>
+      </c>
+      <c r="H46" s="7">
+        <v>3</v>
+      </c>
+      <c r="I46" s="7">
+        <v>8500</v>
+      </c>
+      <c r="J46" s="5">
+        <v>58.5</v>
+      </c>
+      <c r="K46" s="4"/>
+      <c r="L46" s="4"/>
+      <c r="M46" s="7"/>
+      <c r="N46" s="5"/>
+      <c r="O46" s="4"/>
+    </row>
+    <row r="47" spans="1:15">
+      <c r="A47" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B47" s="5"/>
+      <c r="C47" s="5">
+        <v>83.09999999999999</v>
+      </c>
+      <c r="D47" s="4"/>
+      <c r="E47" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F47" s="7">
+        <v>127000</v>
+      </c>
+      <c r="G47" s="7">
+        <v>9000</v>
+      </c>
+      <c r="H47" s="7">
+        <v>3</v>
+      </c>
+      <c r="I47" s="7">
+        <v>15000</v>
+      </c>
+      <c r="J47" s="5">
+        <v>58.5</v>
+      </c>
+      <c r="K47" s="4"/>
+      <c r="L47" s="4"/>
+      <c r="M47" s="7"/>
+      <c r="N47" s="5"/>
+      <c r="O47" s="4"/>
+    </row>
+    <row r="48" spans="1:15">
+      <c r="A48" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B48" s="5"/>
+      <c r="C48" s="5">
+        <v>84.3</v>
+      </c>
+      <c r="D48" s="4"/>
+      <c r="E48" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F48" s="7">
+        <v>120000</v>
+      </c>
+      <c r="G48" s="7">
+        <v>9000</v>
+      </c>
+      <c r="H48" s="7">
+        <v>3</v>
+      </c>
+      <c r="I48" s="7">
+        <v>12500</v>
+      </c>
+      <c r="J48" s="5">
+        <v>58.5</v>
+      </c>
+      <c r="K48" s="4"/>
+      <c r="L48" s="4"/>
+      <c r="M48" s="7"/>
+      <c r="N48" s="5"/>
+      <c r="O48" s="4"/>
+    </row>
+    <row r="49" spans="1:15">
+      <c r="A49" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B49" s="5"/>
+      <c r="C49" s="5">
+        <v>86.90000000000001</v>
+      </c>
+      <c r="D49" s="4"/>
+      <c r="E49" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F49" s="7">
+        <v>154000</v>
+      </c>
+      <c r="G49" s="7">
+        <v>4000</v>
+      </c>
+      <c r="H49" s="7">
+        <v>3</v>
+      </c>
+      <c r="I49" s="7">
+        <v>6500</v>
+      </c>
+      <c r="J49" s="5">
+        <v>58.4</v>
+      </c>
+      <c r="K49" s="4"/>
+      <c r="L49" s="4"/>
+      <c r="M49" s="7"/>
+      <c r="N49" s="5"/>
+      <c r="O49" s="4"/>
+    </row>
+    <row r="50" spans="1:15">
+      <c r="A50" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B50" s="5">
+        <v>9</v>
+      </c>
+      <c r="C50" s="5">
+        <v>86.3</v>
+      </c>
+      <c r="D50" s="4"/>
+      <c r="E50" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F50" s="7">
+        <v>195000</v>
+      </c>
+      <c r="G50" s="7">
+        <v>3000</v>
+      </c>
+      <c r="H50" s="7">
+        <v>3</v>
+      </c>
+      <c r="I50" s="7">
+        <v>6500</v>
+      </c>
+      <c r="J50" s="5">
+        <v>58.1</v>
+      </c>
+      <c r="K50" s="4"/>
+      <c r="L50" s="4"/>
+      <c r="M50" s="7"/>
+      <c r="N50" s="5"/>
+      <c r="O50" s="4"/>
+    </row>
+    <row r="51" spans="1:15">
+      <c r="A51" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B51" s="5"/>
+      <c r="C51" s="5">
+        <v>80.90000000000001</v>
+      </c>
+      <c r="D51" s="4"/>
+      <c r="E51" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F51" s="7">
+        <v>472000</v>
+      </c>
+      <c r="G51" s="7">
+        <v>19000</v>
+      </c>
+      <c r="H51" s="7">
+        <v>3</v>
+      </c>
+      <c r="I51" s="7">
+        <v>17500</v>
+      </c>
+      <c r="J51" s="5">
+        <v>57.9</v>
+      </c>
+      <c r="K51" s="4"/>
+      <c r="L51" s="4"/>
+      <c r="M51" s="7"/>
+      <c r="N51" s="5"/>
+      <c r="O51" s="4"/>
+    </row>
+    <row r="52" spans="1:15">
+      <c r="A52" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B52" s="5"/>
+      <c r="C52" s="5">
+        <v>85.8</v>
+      </c>
+      <c r="D52" s="4"/>
+      <c r="E52" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F52" s="7">
+        <v>270000</v>
+      </c>
+      <c r="G52" s="7">
+        <v>3000</v>
+      </c>
+      <c r="H52" s="7">
+        <v>3</v>
+      </c>
+      <c r="I52" s="7">
+        <v>6500</v>
+      </c>
+      <c r="J52" s="5">
+        <v>57.8</v>
+      </c>
+      <c r="K52" s="4"/>
+      <c r="L52" s="4"/>
+      <c r="M52" s="7"/>
+      <c r="N52" s="5"/>
+      <c r="O52" s="4"/>
+    </row>
+    <row r="53" spans="1:15">
+      <c r="A53" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B53" s="5"/>
+      <c r="C53" s="5">
+        <v>87.09999999999999</v>
+      </c>
+      <c r="D53" s="4"/>
+      <c r="E53" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F53" s="7">
+        <v>131000</v>
+      </c>
+      <c r="G53" s="7">
+        <v>6000</v>
+      </c>
+      <c r="H53" s="7">
+        <v>3</v>
+      </c>
+      <c r="I53" s="7">
+        <v>3500</v>
+      </c>
+      <c r="J53" s="5">
+        <v>57.8</v>
+      </c>
+      <c r="K53" s="4"/>
+      <c r="L53" s="4"/>
+      <c r="M53" s="7"/>
+      <c r="N53" s="5"/>
+      <c r="O53" s="4"/>
+    </row>
+    <row r="54" spans="1:15">
+      <c r="A54" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B54" s="5"/>
+      <c r="C54" s="5">
+        <v>86.3</v>
+      </c>
+      <c r="D54" s="4"/>
+      <c r="E54" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F54" s="7">
+        <v>111000</v>
+      </c>
+      <c r="G54" s="7">
+        <v>8000</v>
+      </c>
+      <c r="H54" s="7">
+        <v>3</v>
+      </c>
+      <c r="I54" s="7">
+        <v>5000</v>
+      </c>
+      <c r="J54" s="5">
+        <v>57.7</v>
+      </c>
+      <c r="K54" s="4"/>
+      <c r="L54" s="4"/>
+      <c r="M54" s="7"/>
+      <c r="N54" s="5"/>
+      <c r="O54" s="4"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:O5"/>
+  <autoFilter ref="A4:O54"/>
   <mergeCells count="2">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="E5" r:id="rId1"/>
+    <hyperlink ref="E6" r:id="rId2"/>
+    <hyperlink ref="E7" r:id="rId3"/>
+    <hyperlink ref="E8" r:id="rId4"/>
+    <hyperlink ref="E9" r:id="rId5"/>
+    <hyperlink ref="E10" r:id="rId6"/>
+    <hyperlink ref="E11" r:id="rId7"/>
+    <hyperlink ref="E12" r:id="rId8"/>
+    <hyperlink ref="E13" r:id="rId9"/>
+    <hyperlink ref="E14" r:id="rId10"/>
+    <hyperlink ref="E15" r:id="rId11"/>
+    <hyperlink ref="E16" r:id="rId12"/>
+    <hyperlink ref="E17" r:id="rId13"/>
+    <hyperlink ref="E18" r:id="rId14"/>
+    <hyperlink ref="E19" r:id="rId15"/>
+    <hyperlink ref="E20" r:id="rId16"/>
+    <hyperlink ref="E21" r:id="rId17"/>
+    <hyperlink ref="E22" r:id="rId18"/>
+    <hyperlink ref="E23" r:id="rId19"/>
+    <hyperlink ref="E24" r:id="rId20"/>
+    <hyperlink ref="E25" r:id="rId21"/>
+    <hyperlink ref="E26" r:id="rId22"/>
+    <hyperlink ref="E27" r:id="rId23"/>
+    <hyperlink ref="E28" r:id="rId24"/>
+    <hyperlink ref="E29" r:id="rId25"/>
+    <hyperlink ref="E30" r:id="rId26"/>
+    <hyperlink ref="E31" r:id="rId27"/>
+    <hyperlink ref="E32" r:id="rId28"/>
+    <hyperlink ref="E33" r:id="rId29"/>
+    <hyperlink ref="E34" r:id="rId30"/>
+    <hyperlink ref="E35" r:id="rId31"/>
+    <hyperlink ref="E36" r:id="rId32"/>
+    <hyperlink ref="E37" r:id="rId33"/>
+    <hyperlink ref="E38" r:id="rId34"/>
+    <hyperlink ref="E39" r:id="rId35"/>
+    <hyperlink ref="E40" r:id="rId36"/>
+    <hyperlink ref="E41" r:id="rId37"/>
+    <hyperlink ref="E42" r:id="rId38"/>
+    <hyperlink ref="E43" r:id="rId39"/>
+    <hyperlink ref="E44" r:id="rId40"/>
+    <hyperlink ref="E45" r:id="rId41"/>
+    <hyperlink ref="E46" r:id="rId42"/>
+    <hyperlink ref="E47" r:id="rId43"/>
+    <hyperlink ref="E48" r:id="rId44"/>
+    <hyperlink ref="E49" r:id="rId45"/>
+    <hyperlink ref="E50" r:id="rId46"/>
+    <hyperlink ref="E51" r:id="rId47"/>
+    <hyperlink ref="E52" r:id="rId48"/>
+    <hyperlink ref="E53" r:id="rId49"/>
+    <hyperlink ref="E54" r:id="rId50"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>